<commit_message>
Lab 3 review fixes: residual value bias note, readable sheet renders, cash chart labels, alternative driver shares
</commit_message>
<xml_diff>
--- a/lab3/out/lab3_budget_tco.xlsx
+++ b/lab3/out/lab3_budget_tco.xlsx
@@ -2614,10 +2614,10 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3391,19 +3391,19 @@
   <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4453,7 +4453,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -5092,15 +5092,15 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Lab 3 review fixes: support versus per building support in A12, scale 85 as Y3 monthly average with review trigger, separate spike prototype and partial A5 check
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lab3/out/lab3_budget_tco.xlsx
+++ b/lab3/out/lab3_budget_tco.xlsx
@@ -2206,7 +2206,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>support 0,25 DevOps + 0,25 BA/PM; change 0,5 Developer + 0,25 QA</t>
+          <t>support 0,25 DevOps + 0,25 BA/PM (чергування, оновлення, онбординг нових будівель); change 0,5 Developer + 0,25 QA</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>однаково для обох сценаріїв</t>
+          <t>однаково для обох сценаріїв; підтримка будівлі (консультації клієнта, перевірка нестабільних лічильників) є змінною витратою 4,80 EUR у COGS ЛР № 1 і в support не дублюється</t>
         </is>
       </c>
     </row>

</xml_diff>